<commit_message>
Import sheet dates as day-month and keep booking search on the live window.
New spreadsheet rows take the next monthly booking ID and warn when the same guest, hotel, and agent already exist. Search stays on the last 30 days plus future trips, and the Sheets backup now includes allotments.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/booking-import-template.xlsx
+++ b/public/templates/booking-import-template.xlsx
@@ -64,8 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,25 +400,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N12"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>5/10/2026</v>
+      <c r="A1" s="1" t="str">
+        <v>5 Oct 26</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -504,8 +505,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>5/10/2026</v>
+      <c r="A3" s="1" t="str">
+        <v>5 Oct 26</v>
       </c>
       <c r="B3" t="str">
         <v>PP</v>
@@ -548,8 +549,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>5/10/2026</v>
+      <c r="A4" s="1" t="str">
+        <v>6 Oct 26</v>
       </c>
       <c r="B4" t="str">
         <v>James Bond</v>

</xml_diff>

<commit_message>
Show Park Fee as Included or Excluded and keep the last sheet column as the guest remark.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/booking-import-template.xlsx
+++ b/public/templates/booking-import-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:O12"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -414,6 +414,7 @@
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,6 +460,9 @@
       <c r="N1" t="str">
         <v/>
       </c>
+      <c r="O1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -492,7 +496,7 @@
         <v>COT</v>
       </c>
       <c r="K2" t="str">
-        <v>Remark</v>
+        <v>Park Fee</v>
       </c>
       <c r="L2" t="str">
         <v>Pick Up</v>
@@ -502,6 +506,9 @@
       </c>
       <c r="N2" t="str">
         <v>VAN</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Remark</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +543,7 @@
         <v>800</v>
       </c>
       <c r="K3" t="str">
-        <v>Excluding National Park Fee</v>
+        <v>EXC</v>
       </c>
       <c r="L3" t="str">
         <v>08:00</v>
@@ -546,6 +553,9 @@
       </c>
       <c r="N3" t="str">
         <v/>
+      </c>
+      <c r="O3" t="str">
+        <v>Arrive 10 min early</v>
       </c>
     </row>
     <row r="4">
@@ -580,7 +590,7 @@
         <v/>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>INC</v>
       </c>
       <c r="L4" t="str">
         <v>07:30</v>
@@ -591,6 +601,9 @@
       <c r="N4" t="str">
         <v/>
       </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -635,6 +648,9 @@
       <c r="N5" t="str">
         <v/>
       </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -679,6 +695,9 @@
       <c r="N6" t="str">
         <v/>
       </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -723,6 +742,9 @@
       <c r="N7" t="str">
         <v/>
       </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -767,6 +789,9 @@
       <c r="N8" t="str">
         <v/>
       </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -811,6 +836,9 @@
       <c r="N9" t="str">
         <v/>
       </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -855,6 +883,9 @@
       <c r="N10" t="str">
         <v/>
       </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -899,6 +930,9 @@
       <c r="N11" t="str">
         <v/>
       </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -943,10 +977,13 @@
       <c r="N12" t="str">
         <v/>
       </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>